<commit_message>
skill v2p2(good,inherit v0p8) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/TBUS_RTM_Generated.xlsx
+++ b/TBUS_RTM_Generated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67917258-459B-443E-B2F7-81A7EDF1A082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1629A76-E346-4FE8-8524-433A3CCA0665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="334">
   <si>
     <t>Test Case List</t>
   </si>
@@ -43,489 +43,496 @@
     <t>TC_001</t>
   </si>
   <si>
-    <t>aplc_clk_freq_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证clk_i时钟频率和单时钟域工作
-配置条件：
-1.配置clk_i为100MHz连续时钟；
-2.配置lane_mode_i=2'b01(4-bit模式)，test_mode_i=1，en_i=1。
+    <t>test_clk_frequency</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. 配置clk_i为100MHz连续时钟
+2. test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)
+3. 外部CSR File已实现VERSION(0x00)、CTRL(0x04)、STATUS(0x08)、LAST_ERR(0x0C)寄存器
 输入激励：
-1.驱动clk_i持续运行，依次发送WR_CSR(0x10)/RD_CSR(0x11)/AHB_WR32(0x20)/AHB_RD32(0x21)命令帧；
-2.使用频率计测量clk_i实际频率。
+1. 驱动clk_i持续运行，发送WR_CSR(0x10)命令帧：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+2. 发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00
+3. 发送AHB_WR32(0x20)命令帧：opcode=0x20, addr=0x00000100, wdata=0xDEADBEEF
+4. 发送AHB_RD32(0x21)命令帧：opcode=0x21, addr=0x00000100
 期望结果：
-1.所有内部逻辑在clk_i上升沿正确同步，协议接收、状态机控制和AHB-Lite主接口同域工作，无跨时钟域问题；
-2.模块在100MHz目标频率下正常工作，所有时序满足约束。
+1. 所有内部逻辑在clk_i上升沿正确同步，协议接收、状态机控制和AHB-Lite主接口同域工作，无跨时钟域问题
+2. 模块在100MHz目标频率下正常工作，所有时序满足约束
+3. 四类命令均正确执行并返回STS_OK(0x00)
+coverage check点：
+1. 收集clk_i频率在不同操作下的稳定性覆盖率
+2. 收集各命令在100MHz下的端到端延时分布</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>test_reset_behavior</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni连接复位源，模块处于任意工作状态
+2. test_mode_i=1，en_i=1，lane_mode_i=2'b01
+3. 模块正在执行AHB_WR32命令期间触发复位
+输入激励：
+1. rst_ni拉低触发异步复位（模块正在执行命令期间）
+2. 释放rst_ni（同步释放），等待若干clk_i周期
+3. 检查前端FSM状态front_state和后端FSM状态back_state
+4. 检查所有输出端口：pdo_oe_o, htrans_o, csr_rd_en_o, csr_wr_en_o, pdo_o
+5. 复位后重新初始化：test_mode_i=1, en_i=1, lane_mode_i=2'b01
+6. 发送RD_CSR(0x11)命令帧验证模块恢复正常工作
+期望结果：
+1. rst_ni下降沿立即触发复位，无需等待clk_i上升沿
+2. rst_ni释放时在clk_i上升沿同步退出复位
+3. 复位后front_state=IDLE(3'd0), back_state=S_IDLE(3'd0)，所有协议/响应上下文清空
+4. 复位后pdo_oe_o=0, htrans_o=2'b00(IDLE), csr_rd_en_o=0, csr_wr_en_o=0, pdo_o=4'b0
+5. 复位后重新发送命令可正常执行并返回STS_OK(0x00)
+coverage check点：
+1. 收集复位在不同FSM状态下触发的情况
+2. 收集复位后输出端口deassert的时序覆盖率</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>test_csr_write_read</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成（同步释放后）
+2. test_mode_i=1（测试模式使能）
+3. en_i=1（模块使能）
+4. lane_mode_i=2'b01（4-bit模式）
+5. 外部CSR File已实现VERSION(0x00)、CTRL(0x04)、STATUS(0x08)、LAST_ERR(0x0C)寄存器
+输入激励：
+1. 发送WR_CSR(0x10)命令帧写CTRL(0x04)：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+   - 帧结构：[0x10(8bit) | 0x04(8bit) | wdata(32bit)] = 48bit
+   - 4-bit模式需12个clk_i周期接收
+2. 发送RD_CSR(0x11)命令帧读VERSION(0x00)：opcode=0x11, reg_addr=0x00
+   - 帧结构：[0x11(8bit) | 0x00(8bit)] = 16bit
+   - 4-bit模式需4个clk_i周期接收
+3. 发送RD_CSR(0x11)命令帧读CTRL(0x04)：opcode=0x11, reg_addr=0x04
+4. 发送WR_CSR(0x10)命令帧写STATUS(0x08)：opcode=0x10, reg_addr=0x08, wdata=0x00000000
+5. 发送RD_CSR(0x11)命令帧读LAST_ERR(0x0C)：opcode=0x11, reg_addr=0x0C
+期望结果：
+1. WR_CSR执行：csr_wr_en_o脉冲持续1个clk_i周期，同周期csr_addr_o=0x04, csr_wdata_o=0x00000001有效；返回pdo_o[7:0]=STS_OK(0x00)
+2. RD_CSR执行：csr_rd_en_o脉冲持续1个clk_i周期；下一周期外部CSR File驱动csr_rdata_i[31:0]；返回pdo_o[39:0]=[STS_OK(0x00) | rdata(32bit)]
+3. 所有CSR写操作返回STS_OK(0x00)，响应8bit状态码
+4. 所有CSR读操作返回STS_OK(0x00)+rdata[31:0]，响应40bit(status8+rdata32)
+coverage check点：
+1. 遍历所有CSR寄存器地址(0x00~0x3F)的功能覆盖率
+2. 收集csr_addr_o的功能覆盖率
+3. 收集wdata和rdata的数据覆盖率</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>test_csr_addr_boundary</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
+输入激励：
+1. 发送RD_CSR(0x11)命令帧，reg_addr=0x3F（边界内最大有效地址）：opcode=0x11, reg_addr=0x3F
+2. 发送RD_CSR(0x11)命令帧，reg_addr=0x40（边界外最小无效地址）：opcode=0x11, reg_addr=0x40
+3. 发送WR_CSR(0x10)命令帧，reg_addr=0x40：opcode=0x10, reg_addr=0x40, wdata=0xAAAAAAAA
+4. 发送RD_CSR(0x11)命令帧，reg_addr=0xFF：opcode=0x11, reg_addr=0xFF
+5. 发送WR_CSR(0x10)命令帧，reg_addr=0x00（有效地址）：opcode=0x10, reg_addr=0x00, wdata=0x12345678
+期望结果：
+1. reg_addr=0x3F：正常发起CSR读，csr_rd_en_o=1，返回STS_OK(0x00)+rdata
+2. reg_addr=0x40：前置检查拒绝，返回STS_BAD_REG(0x10)，不发起CSR读操作(csr_rd_en_o=0)
+3. reg_addr=0x40 WR_CSR：前置检查拒绝，返回STS_BAD_REG(0x10)，不发起CSR写操作(csr_wr_en_o=0)
+4. reg_addr=0xFF：前置检查拒绝，返回STS_BAD_REG(0x10)，不发起CSR操作
+5. reg_addr=0x00：正常发起CSR写，csr_wr_en_o=1，返回STS_OK(0x00)
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
   </si>
   <si>
-    <t>TC_002</t>
-  </si>
-  <si>
-    <t>aplc_reset_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证rst_n_i异步复位与同步释放及复位后状态
-配置条件：
-1.配置clk_i=100MHz，lane_mode_i=2'b01，test_mode_i=1，en_i=1；
-2.模块处于正常工作状态（已发送若干命令）。
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>test_mode_control</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.在任意工作状态下拉低rst_n_i触发异步复位；
-2.释放rst_n_i（同步释放）；
-3.检查front_state、back_state及所有输出端口。
+1. 设置test_mode_i=0, en_i=1，发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00
+2. 检查csr_rd_en_o和htrans_o是否为0
+3. 设置test_mode_i=1, en_i=0，发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00
+4. 检查csr_rd_en_o和htrans_o是否为0
+5. 设置test_mode_i=1, en_i=1，发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00
+6. 检查命令正常执行
 期望结果：
-1.rst_n_i下降沿立即触发复位；释放时在clk_i上升沿同步退出复位；
-2.复位后front_state=IDLE(3'd0)，back_state=S_IDLE(3'd0)；
-3.pdo_oe_o=0，htrans_o=2'b00(IDLE)，csr_rd_en_o=0，csr_wr_en_o=0，pdo_o=4'b0；LANE_MODE恢复默认1-bit模式。
+1. test_mode_i=0：前置检查检测到test_mode_i=0，返回STS_NOT_IN_TEST(0x04)；不发起CSR/AHB访问(csr_rd_en_o=0, htrans_o=IDLE)
+2. en_i=0：前置检查检测到en_i=0，返回STS_DISABLED(0x08)；不发起CSR/AHB访问
+3. test_mode_i=1, en_i=1：前置检查通过，正常执行命令并返回STS_OK(0x00)+rdata
+coverage check点：
+1. 收集test_mode_i=0/1和en_i=0/1的组合覆盖率
+2. 收集STS_NOT_IN_TEST和STS_DISABLED状态码的功能覆盖率</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>test_lane_mode</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1
+输入激励：
+1. 配置lane_mode_i=2'b00(1-bit模式)，发送WR_CSR(0x10)命令帧：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+   - 1-bit模式：每拍收发1bit，帧长48bit需48个clk_i周期接收
+2. 发送AHB_RD32(0x21)命令帧：opcode=0x21, addr=0x00000100
+   - 1-bit模式：帧长40bit需40个clk_i周期接收
+3. 配置lane_mode_i=2'b01(4-bit模式)，发送WR_CSR(0x10)命令帧：opcode=0x10, reg_addr=0x04, wdata=0x00000002
+   - 4-bit模式：每拍收发4bit，帧长48bit需12个clk_i周期接收
+4. 发送AHB_RD32(0x21)命令帧：opcode=0x21, addr=0x00000100
+   - 4-bit模式：帧长40bit需10个clk_i周期接收
+期望结果：
+1. 1-bit模式：仅pdi_i[0]有效，其余位忽略；每拍收发1bit；命令执行正确
+2. 4-bit模式：pdi_i[3:0]均有效；每拍收发4bit；命令执行正确
+3. 两种模式下MSB-first顺序传输均正确
+4. 两种模式下命令均返回STS_OK(0x00)，读命令返回正确rdata
+coverage check点：
+1. 收集lane_mode_i=2'b00和2'b01的功能覆盖率
+2. 收集1-bit和4-bit模式下各命令的执行覆盖率</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>test_protocol_frame</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
+输入激励：
+1. pcs_ni拉低开启事务，发送完整WR_CSR(0x10)命令帧(48bit)，pcs_ni拉高结束事务
+2. pcs_ni拉低，发送完整RD_CSR(0x11)命令帧(16bit)，pcs_ni拉高
+3. pcs_ni拉低，发送完整AHB_WR32(0x20)命令帧(72bit)，pcs_ni拉高
+4. pcs_ni拉低，发送完整AHB_RD32(0x21)命令帧(40bit)，pcs_ni拉高
+5. pcs_ni拉低，发送WR_CSR帧，在rx_count&lt;expected_rx_bits时提前将pcs_ni拉高（opcode已锁存）
+6. 命令执行完成后观测pdo_oe_o和pdo_o的时序
+期望结果：
+1. pcs_ni=1时空闲；pcs_ni=0时开启帧接收；pcs_ni拉高时结束事务
+2. 1-bit模式仅bit0有效，4-bit模式全部4位有效；MSB-first传输
+3. 响应阶段pdo_oe_o=1，模块驱动pdo_o输出；非发送阶段pdo_oe_o=0
+4. 四类命令帧长正确：WR_CSR 48bit, RD_CSR 16bit, AHB_WR32 72bit, AHB_RD32 40bit
+5. 帧中止(frame_abort)：返回STS_FRAME_ERR(0x01)，不发起CSR/AHB访问
+6. 请求-响应间固定1个clk_i周期turnaround，turnaround期间pdo_oe_o=0，TX阶段pdo_oe_o=1
+coverage check点：
+1. 收集四类命令帧格式的功能覆盖率
+2. 收集frame_abort在不同接收进度下的覆盖率
+3. 收集turnaround时序的覆盖率</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>test_opcode_decode</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
+输入激励：
+1. 发送opcode=0x10(WR_CSR)命令帧：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+2. 发送opcode=0x11(RD_CSR)命令帧：opcode=0x11, reg_addr=0x00
+3. 发送opcode=0x20(AHB_WR32)命令帧：opcode=0x20, addr=0x00000100, wdata=0xDEADBEEF
+4. 发送opcode=0x21(AHB_RD32)命令帧：opcode=0x21, addr=0x00000100
+5. 发送opcode=0xFF(非法值)命令帧
+6. 发送opcode=0x00(非法值)命令帧
+7. 发送opcode=0x30(非法值)命令帧
+期望结果：
+1. 有效opcode(0x10/0x11/0x20/0x21)：前端收满8bit后锁存opcode，根据opcode确定expected_rx_bits，正确发起对应类型任务
+2. 非法opcode(0xFF/0x00/0x30)：前置检查检测到非法opcode，返回STS_BAD_OPCODE(0x02)，不发起CSR/AHB访问
+3. 有效命令正常执行并返回对应状态码和数据
+coverage check点：
+1. 收集有效opcode(0x10/0x11/0x20/0x21)的功能覆盖率
+2. 收集非法opcode值的交叉覆盖率</t>
+  </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>test_ctrl_config</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1
+输入激励：
+1. 通过WR_CSR(0x10)写CTRL(0x04)寄存器：EN=1, LANE_MODE=2'b00(1-bit)：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+2. 发送RD_CSR(0x11)读回CTRL(0x04)验证：opcode=0x11, reg_addr=0x04
+3. 通过WR_CSR(0x10)写CTRL(0x04)寄存器：LANE_MODE=2'b01(4-bit)：opcode=0x10, reg_addr=0x04, wdata=0x00000002
+4. 发送RD_CSR(0x11)读回CTRL(0x04)验证：opcode=0x11, reg_addr=0x04
+5. 通过WR_CSR(0x10)写CTRL(0x04)寄存器：SOFT_RST=1：opcode=0x10, reg_addr=0x04, wdata含SOFT_RST位
+6. 检查SOFT_RST写1后协议上下文清零并恢复默认lane模式
+期望结果：
+1. LANE_MODE=2'b00对应1-bit模式，01对应4-bit模式
+2. 读回CTRL寄存器值与写入值一致
+3. SOFT_RST写1触发协议上下文清零并恢复默认lane模式(1-bit)
+4. 所有CSR写操作返回STS_OK(0x00)
+coverage check点：
+1. 收集CTRL.EN, CTRL.LANE_MODE, CTRL.SOFT_RST字段组合的功能覆盖率
+2. 收集SOFT_RST触发后的状态恢复覆盖率</t>
+  </si>
+  <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>test_lane_mode_switch</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1
+输入激励：
+1. 配置lane_mode_i=2'b01(4-bit模式)
+2. pcs_ni拉低开始事务，发送WR_CSR(0x10)命令帧(48bit)
+3. 在事务执行期间(pcs_ni=0)将lane_mode_i从2'b01切换为2'b00
+4. pcs_ni拉高结束事务，观测响应
+5. 复位模块，配置lane_mode_i=2'b01
+6. pcs_ni=1(空闲态)时将lane_mode_i切换为2'b00
+7. pcs_ni拉低开始新事务，发送WR_CSR(0x10)命令帧
+期望结果：
+1. 事务期间切换lane_mode_i：bpc(移位宽度)立即改变，帧数据错位；模块不检测此违规
+2. 帧数据损坏可能误触发STS_BAD_OPCODE(0x02)或STS_FRAME_ERR(0x01)
+3. 空闲态切换lane_mode_i：新事务使用更新后的lane_mode；帧数据正确无错位
+4. 空闲态切换后命令正常执行并返回STS_OK(0x00)
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
   </si>
   <si>
-    <t>TC_003</t>
-  </si>
-  <si>
-    <t>aplc_csr_write_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证WR_CSR(0x10)命令写CSR寄存器功能
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.模块解复位，进入正常工作状态。
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>test_no_interrupt</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.依次发送WR_CSR(0x10)命令写VERSION(0x00)、CTRL(0x04)、STATUS(0x08)、LAST_ERR(0x0C)，写入随机数据；
-2.观测csr_wr_en_o、csr_addr_o、csr_wdata_o信号。
+1. 发送RD_CSR(0x11)命令帧触发正常完成事件，检查是否有IRQ信号
+2. 发送opcode=0xFF触发STS_BAD_OPCODE错误，检查是否有IRQ信号
+3. 发送WR_CSR帧后提前拉高pcs_ni触发STS_FRAME_ERR错误，检查是否有IRQ信号
+4. 连续发送3条错误命令(opcode=0xFF, reg_addr=0x40, addr非对齐)，每条命令后读取STATUS(0x08)和LAST_ERR(0x0C)寄存器
 期望结果：
-1.csr_wr_en_o脉冲持续1周期；同周期csr_addr_o和csr_wdata_o有效；
-2.外部CSR File采样写入数据；写操作返回STS_OK(0x00)。
+1. MVP版本不实现独立中断输出，无IRQ信号拉高
+2. 错误信息通过STATUS寄存器和LAST_ERR寄存器查询，采用轮询方式获取
+3. 每次错误状态通过响应帧8bit状态码直接返回给ATE
+4. 前一条错误信息被新命令覆盖，ATE应每条命令后检查状态码
 coverage check点：
-对CSR写地址(0x00/0x04/0x08/0x0C)和写数据位宽收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_004</t>
-  </si>
-  <si>
-    <t>aplc_csr_read_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证RD_CSR(0x11)命令读CSR寄存器功能
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.先通过WR_CSR(0x10)写入已知数据到VERSION(0x00)、CTRL(0x04)。
+1. 收集各类错误事件的STATUS和LAST_ERR寄存器值覆盖率
+2. 收集连续错误覆盖率的时序覆盖率</t>
+  </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>test_error_handling</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
+3. AHB从设备已连接，可返回hresp_i=1或延迟hready_i
 输入激励：
-1.发送RD_CSR(0x11)命令读VERSION(0x00)、CTRL(0x04)；
-2.观测csr_rd_en_o、csr_rdata_i和响应帧RDATA。
+1. [FRAME_ERR] 发送WR_CSR帧，pcs_ni在rx_count&lt;expected_rx_bits时提前拉高（opcode已锁存）
+2. [BAD_OPCODE] 发送opcode=0xFF命令帧
+3. [NOT_IN_TEST] 设置test_mode_i=0，发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00；测试完成后恢复test_mode_i=1
+4. [DISABLED] 设置en_i=0，发送RD_CSR(0x11)命令帧：opcode=0x11, reg_addr=0x00；测试完成后恢复en_i=1
+5. [BAD_REG] 发送RD_CSR(0x11)命令帧，reg_addr=0x40：opcode=0x11, reg_addr=0x40
+6. [ALIGN_ERR] 发送AHB_WR32(0x20)命令帧，addr=0x00000101(addr[1:0]=2'b01)：opcode=0x20, addr=0x00000101, wdata=0xDEADBEEF
+7. [AHB_ERR-hresp] 发送AHB_WR32(0x20)命令帧，从设备返回hresp_i=1：opcode=0x20, addr=0x00000100, wdata=0xDEADBEEF
+8. [AHB_ERR-timeout] 发送AHB_RD32(0x21)命令帧，hready_i持续为0超过256周期：opcode=0x21, addr=0x00000100
 期望结果：
-1.csr_rd_en_o脉冲持续1周期；下一周期外部CSR File将读数据稳定在csr_rdata_i上；
-2.模块正确采样csr_rdata_i；读操作返回STS_OK(0x00)+RDATA[31:0]，RDATA与写入值一致。
+1. STS_FRAME_ERR(0x01)：frame_abort产生，不发起CSR/AHB访问
+2. STS_BAD_OPCODE(0x02)：前置检查失败，不发起CSR/AHB访问
+3. STS_NOT_IN_TEST(0x04)：test_mode_i=0时拒绝，不发起CSR/AHB访问
+4. STS_DISABLED(0x08)：en_i=0时拒绝，不发起CSR/AHB访问
+5. STS_BAD_REG(0x10)：reg_addr&gt;=0x40时拒绝，csr_rd_en_o=0
+6. STS_ALIGN_ERR(0x20)：addr[1:0]!=2'b00时拒绝，不发起AHB访问(htrans_o保持IDLE)
+7. STS_AHB_ERR(0x40)-hresp：STATE_WAIT检测到hresp_i=1，转STATE_ERR
+8. STS_AHB_ERR(0x40)-timeout：timeout_cnt_q递增至255触发STATE_ERR
 coverage check点：
-对CSR读地址和1周期读延迟时序收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_005</t>
-  </si>
-  <si>
-    <t>aplc_csr_bad_addr_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证非法CSR地址(&gt;=0x40)的前置拒绝
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
+1. 收集所有8种状态码(0x00/0x01/0x02/0x04/0x08/0x10/0x20/0x40)的功能覆盖率
+2. 收集AHB错误类型(hresp_i=1 vs timeout)的交叉覆盖率</t>
+  </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>test_error_priority</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.发送WR_CSR(0x10)命令，reg_addr随机取0x40、0x5F、0xFF等&gt;=0x40的地址；
-2.发送RD_CSR(0x11)命令，reg_addr随机取0x40、0x7F、0xFF等&gt;=0x40的地址；
-3.观测csr_wr_en_o、csr_rd_en_o信号。
+1. 设置test_mode_i=0, en_i=0，发送RD_CSR(0x11)命令帧同时满足NOT_IN_TEST和DISABLED：opcode=0x11, reg_addr=0x00
+2. 复位后设置test_mode_i=1, en_i=0，发送RD_CSR(0x11)命令帧reg_addr=0x40（同时满足DISABLED和BAD_REG）：opcode=0x11, reg_addr=0x40
+3. 复位后设置test_mode_i=1, en_i=1，发送AHB_WR32(0x20)命令帧addr=0x00000101（仅ALIGN_ERR）：opcode=0x20, addr=0x00000101, wdata=0xDEADBEEF
+4. 复位后设置test_mode_i=1, en_i=1，发送opcode=0xFF命令帧（仅BAD_OPCODE）
+5. 发送WR_CSR帧提前拉高pcs_ni（同时满足FRAME_ERR和BAD_OPCODE）：opcode在锁存后截断帧
 期望结果：
-1.所有非法地址命令返回STS_BAD_REG(0x10)；
-2.csr_wr_en_o=0，csr_rd_en_o=0，不发起CSR访问。
+1. NOT_IN_TEST+DISABLED同时满足：返回STS_NOT_IN_TEST(0x04)（优先级更高）
+2. DISABLED+BAD_REG同时满足：返回STS_DISABLED(0x08)（优先级更高）
+3. 仅ALIGN_ERR：返回STS_ALIGN_ERR(0x20)
+4. 仅BAD_OPCODE：返回STS_BAD_OPCODE(0x02)
+5. FRAME_ERR+BAD_OPCODE同时满足：返回STS_FRAME_ERR(0x01)（最高优先级）
+6. 每次仅报告一个状态码，按固定优先级链：FRAME_ERR(0x01)&gt;BAD_OPCODE(0x02)&gt;NOT_IN_TEST(0x04)&gt;DISABLED(0x08)&gt;BAD_REG(0x10)&gt;ALIGN_ERR(0x20)
 coverage check点：
-对reg_addr&gt;=0x40的地址边界值收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_006</t>
-  </si>
-  <si>
-    <t>aplc_mode_gate_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证test_mode_i和en_i前置门控行为
-配置条件：
-1.配置clk_i=100MHz，lane_mode_i=2'b01(4-bit模式)。
+1. 收集多错误组合场景的功能覆盖率
+2. 收集优先级链各节点的状态码覆盖率</t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>test_performance_latency</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1
+3. hready_i=1(零等待)
 输入激励：
-1.test_mode_i=0, en_i=1时，发送RD_CSR(0x11)有效命令帧；
-2.test_mode_i=1, en_i=0时，发送WR_CSR(0x10)有效命令帧；
-3.test_mode_i=1, en_i=1时，发送WR_CSR(0x10)/RD_CSR(0x11)/AHB_WR32(0x20)/AHB_RD32(0x21)四类命令。
+1. [4-bit AHB_RD32] 配置lane_mode_i=2'b01，发送AHB_RD32(0x21)命令帧：opcode=0x21, addr=0x00000100
+   测量端到端延时：请求接收10cyc + 译码1~2cyc + AHB返回1cyc + turnaround 1cyc + 响应发送10cyc
+2. [4-bit AHB_WR32] 发送AHB_WR32(0x20)命令帧：opcode=0x20, addr=0x00000100, wdata=0xDEADBEEF
+   测量端到端延时：请求接收18cyc + 执行2cyc + turnaround 1cyc + 响应发送2cyc
+3. [1-bit AHB_RD32] 配置lane_mode_i=2'b00，发送AHB_RD32(0x21)命令帧
+   测量端到端延时：请求接收40cyc + 译码1~2cyc + AHB返回1cyc + turnaround 1cyc + 响应发送40cyc
+4. [1-bit WR_CSR] 发送WR_CSR(0x10)命令帧：opcode=0x10, reg_addr=0x04, wdata=0x00000001
+   测量端到端延时：请求接收48cyc + 执行~6cyc + turnaround 1cyc + 响应发送8cyc
+5. [AHB超时] 发送AHB_RD32(0x21)命令帧，hready_i持续为0超过256周期
+   检查9-bit计数器在STATE_WAIT递增至255触发STATE_ERR
 期望结果：
-1.test_mode_i=0时返回STS_NOT_IN_TEST(0x04)，不发起CSR/AHB访问；
-2.en_i=0时返回STS_DISABLED(0x08)，不发起CSR/AHB访问；
-3.test_mode_i=1且en_i=1时，前置检查通过，正常执行命令并返回正确状态码和数据。
+1. 4-bit AHB_RD32最小延时约23~24 cycles
+2. 4-bit AHB_WR32最小延时约23 cycles
+3. 1-bit AHB_RD32最小延时约83~84 cycles
+4. 1-bit WR_CSR最小延时约63 cycles
+5. AHB超时：9-bit计数器在STATE_WAIT递增至BUS_TIMEOUT_CYCLES-1(默认255)触发STATE_ERR，返回STS_AHB_ERR(0x40)
 coverage check点：
-对test_mode_i和en_i的0/1组合收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_007</t>
-  </si>
-  <si>
-    <t>aplc_lane_mode_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证1-bit和4-bit通道模式切换
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1。
+1. 收集各命令在1-bit和4-bit模式下的端到端延时分布
+2. 收集AHB等待周期数的覆盖率</t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>test_dfx_observability</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. 仿真/调试环境，内部调试信号可观测
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.lane_mode_i=2'b00(1-bit模式)时，发送WR_CSR(0x10)和AHB_RD32(0x21)命令；
-2.lane_mode_i=2'b01(4-bit模式)时，发送WR_CSR(0x10)和AHB_RD32(0x21)命令；
-3.对比两种模式的帧接收周期。
+1. 发送WR_CSR(0x10)命令帧，观测内部调试信号：front_state, back_state, opcode, addr, wdata, rdata, status_code, rx_count, tx_count, lane_mode
+2. 发送AHB_RD32(0x21)命令帧，观测内部调试信号
+3. 发送opcode=0xFF非法命令，观测front_state跳转和status_code变化
+4. 发送WR_CSR帧后提前拉高pcs_ni，观测frame_abort和rx_count值
 期望结果：
-1.1-bit模式每拍收发1bit(pdi_i[0])，帧接收周期为帧长bit数；
-2.4-bit模式每拍收发4bit(pdi_i[3:0])，帧接收周期为帧长/4；
-3.两种模式命令执行结果一致。
-coverage check点：
-对lane_mode_i的2'b00和2'b01配置收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_008</t>
-  </si>
-  <si>
-    <t>aplc_frame_recv_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证四类命令帧的完整接收和响应格式
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.发送WR_CSR(0x10)命令帧(48bit: opcode8+reg_addr8+wdata32)；
-2.发送RD_CSR(0x11)命令帧(16bit: opcode8+reg_addr8)；
-3.发送AHB_WR32(0x20)命令帧(72bit: opcode8+addr32+wdata32)；
-4.发送AHB_RD32(0x21)命令帧(40bit: opcode8+addr32)；
-5.在1-bit模式下重复上述命令。
-期望结果：
-1.每类命令帧接收完成后产生frame_valid；
-2.WR_CSR/AHB_WR32响应8bit状态码；RD_CSR/AHB_RD32响应40bit(8bit状态+32bit读数据)；
-3.pcs_n_i=1时空闲；pcs_n_i=0时开启帧接收；pcs_n_i拉高时结束事务；
-4.1-bit模式仅pdi_i[0]有效；4-bit模式pdi_i[3:0]均有效；MSB-first顺序传输；
-5.响应阶段pdo_oe_o=1驱动pdo_o；非发送阶段pdo_oe_o=0。
-coverage check点：
-对四类opcode(0x10/0x11/0x20/0x21)和两种lane模式收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_009</t>
-  </si>
-  <si>
-    <t>aplc_frame_abort_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证帧中止(frame_abort)行为
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.发送WR_CSR(0x10)帧，在rx_count&lt;expected_rx_bits时提前将pcs_n_i拉高；
-2.发送AHB_WR32(0x20)帧，仅发送部分opcode后提前将pcs_n_i拉高；
-3.在1-bit模式下重复帧中止场景。
-期望结果：
-1.产生frame_abort，返回STS_FRAME_ERR(0x01)；
-2.不发起CSR/AHB访问。
-coverage check点：
-对帧中止时的rx_count值范围收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_010</t>
-  </si>
-  <si>
-    <t>aplc_turnaround_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证请求-响应之间的turnaround周期
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.发送WR_CSR(0x10)命令，观测请求阶段结束到响应阶段开始的时序；
-2.发送RD_CSR(0x11)命令，观测turnaround周期；
-3.发送AHB_WR32(0x20)/AHB_RD32(0x21)命令，观测turnaround周期。
-期望结果：
-1.请求阶段与响应阶段之间固定插入1个clk_i周期turnaround；
-2.turnaround期间pdo_oe_o=0；TX阶段pdo_oe_o=1。
+1. 可观测front_state状态机跳转：IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE
+2. 可观测back_state状态机跳转：S_IDLE→S_LOAD_TASK→S_EXEC→S_WAIT_AHB→S_BUILD_RESP→S_DONE
+3. 可观测opcode值(0x10/0x11/0x20/0x21/0xFF)
+4. 可观测addr、wdata、rdata数据通路
+5. 可观测status_code(0x00/0x01/0x02等)
+6. 可观测rx_count和tx_count计数器值
+7. 便于波形定位和故障复现
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
   </si>
   <si>
-    <t>TC_011</t>
-  </si>
-  <si>
-    <t>aplc_opcode_valid_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证合法opcode解析和帧长度确定
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>test_memory_map</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. SoC集成环境
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.依次发送opcode为0x10(WR_CSR)、0x11(RD_CSR)、0x20(AHB_WR32)、0x21(AHB_RD32)的完整命令帧；
-2.观测前端FSM状态和expected_rx_bits值。
+1. 检查模块CSR是否出现在AHB memory map中
+2. 发送AHB_WR32(0x20)命令帧访问addr=0x00000100：opcode=0x20, addr=0x00000100, wdata=0xCAFEBABE
+3. 发送AHB_RD32(0x21)命令帧访问addr=0x00000100：opcode=0x21, addr=0x00000100
+4. 发送AHB_WR32(0x20)命令帧访问addr=0x00000200：opcode=0x20, addr=0x00000200, wdata=0x12345678
+5. 发送AHB_RD32(0x21)命令帧访问addr=0x00000200：opcode=0x21, addr=0x00000200
 期望结果：
-1.前端收满8bit后锁存opcode；
-2.0x10对应48bit、0x11对应16bit、0x20对应72bit、0x21对应40bit；
-3.正确发起对应类型任务。
+1. 模块CSR不进入SoC AHB memory map，仅通过协议命令(WR_CSR/RD_CSR)访问
+2. AHB Master采用32bit地址空间和word(32-bit)访问粒度
+3. 写后读数据一致：addr=0x00000100读回0xCAFEBABE，addr=0x00000200读回0x12345678
+4. 具体可达目标地址范围由SoC顶层统一约束
 coverage check点：
-对四类合法opcode收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_012</t>
-  </si>
-  <si>
-    <t>aplc_opcode_invalid_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证非法opcode检测
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
+1. 收集AHB地址空间的功能覆盖率
+2. 收集AHB写后读一致性的覆盖率</t>
+  </si>
+  <si>
+    <t>TC_017</t>
+  </si>
+  <si>
+    <t>test_ahb_protocol</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. test_mode_i=1, en_i=1, lane_mode_i=2'b01(4-bit模式)
+3. AHB从设备已连接，hready_i=1(零等待)
 输入激励：
-1.发送opcode为0x00、0xFF、0x30、0x12等不在{0x10,0x11,0x20,0x21}中的完整帧；
-2.发送opcode为0x10/0x11/0x20/0x21的部分位翻转值。
+1. [AHB写2-phase] 发送AHB_WR32(0x20)命令帧：opcode=0x20, addr=0x00000100, wdata=0xDEADBEEF
+   观测T1(STATE_REQ): haddr_o=0x00000100, hwrite_o=1, htrans_o=NONSEQ(2'b10)
+   观测T2(STATE_WAIT): htrans_o=IDLE(2'b00), hwdata_o=0xDEADBEEF
+2. [AHB读2-phase] 发送AHB_RD32(0x21)命令帧：opcode=0x21, addr=0x00000100
+   观测T1(STATE_REQ): haddr_o=0x00000100, hwrite_o=0, htrans_o=NONSEQ(2'b10)
+   观测T2(STATE_WAIT): htrans_o=IDLE, hrdata_i有效时采样
+3. [固定信号] 检查hsize_o=3'b010(WORD), hburst_o=3'b000(SINGLE)
+4. [htrans时序] 检查htrans_o仅在STATE_REQ驱动NONSEQ(2'b10)持续1周期，其余时刻均为IDLE(2'b00)
+5. [AHB错误恢复] 构造hresp_i=1的AHB读命令，观察STATE_ERR后自动恢复STATE_IDLE
+6. 观测AHB错误后模块可立即接受新请求
 期望结果：
-1.前置检查检测到非法opcode，返回STS_BAD_OPCODE(0x02)；
-2.不发起CSR/AHB访问。
+1. AHB写T1/T2错开1拍：haddr与hwdata不在同一拍
+2. AHB读T1/T2正确：haddr在T1驱动，hrdata在T2采样
+3. hsize_o固定3'b010(WORD), hburst_o固定3'b000(SINGLE)
+4. htrans_o仅在STATE_REQ为NONSEQ(2'b10)持续1周期，其余为IDLE(2'b00)
+5. STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans=IDLE, haddr=0
+6. 错误恢复后模块可立即接受新请求，无需外部干预
 coverage check点：
-对非法opcode的取值范围收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_013</t>
-  </si>
-  <si>
-    <t>aplc_ctrl_config_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证CTRL寄存器EN/LANE_MODE/SOFT_RST配置和lane切换行为
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1。
+1. 收集AHB 2-phase时序的功能覆盖率
+2. 收集htrans_o在各FSM状态下的值覆盖率
+3. 收集AHB错误恢复的覆盖率</t>
+  </si>
+  <si>
+    <t>TC_018</t>
+  </si>
+  <si>
+    <t>test_low_power</t>
+  </si>
+  <si>
+    <t>配置条件：
+1. rst_ni释放完成
+2. lane_mode_i=2'b01(4-bit模式)
 输入激励：
-1.通过WR_CSR(0x10)写CTRL(0x04)，配置EN=1，LANE_MODE=2'b00(1-bit)；
-2.通过WR_CSR(0x10)写CTRL(0x04)，配置EN=1，LANE_MODE=2'b01(4-bit)；
-3.通过WR_CSR(0x10)写CTRL(0x04)，配置SOFT_RST=1，观测协议上下文清零；
-4.pcs_n_i=0(事务期间)改变lane_mode_i，观察帧数据错位；
-5.pcs_n_i=1(空闲态)改变lane_mode_i，然后发起新事务。
+1. [空闲态翻转] 模块空闲态(pcs_ni=1)，观测接收移位寄存器(rx_shift_q)、发送移位寄存器、超时计数器是否更新
+2. [非测试模式AHB输出] 设置test_mode_i=0，观测htrans_o是否保持IDLE(2'b00)
+3. [无有效任务AHB输出] 设置test_mode_i=1, en_i=0，观测htrans_o是否保持IDLE(2'b00)
+4. [超时计数器] 发送AHB_WR32(0x20)命令帧使模块进入STATE_WAIT，观测超时计数器递增；结束后检查STATE_REQ时清零；空闲态不工作
 期望结果：
-1.LANE_MODE=2'b00对应1-bit模式，2'b01对应4-bit模式；
-2.SOFT_RST写1触发协议上下文清零并恢复默认lane模式；
-3.事务期间切换lane_mode_i导致移位宽度变化、帧数据错位；
-4.空闲态切换后新事务使用更新后的lane模式，帧数据正确。
+1. 空闲态：接收移位寄存器不更新，发送移位寄存器不翻转，超时计数器不工作
+2. test_mode_i=0时：htrans_o保持IDLE(2'b00)，无AHB总线翻转
+3. en_i=0时：htrans_o保持IDLE(2'b00)，无AHB总线翻转
+4. 超时计数器仅在STATE_WAIT期间递增，STATE_REQ时清零，IDLE态不工作
 coverage check点：
-对CTRL.EN/LANE_MODE/SOFT_RST字段的配置组合收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_014</t>
-  </si>
-  <si>
-    <t>aplc_status_polling_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证MVP无中断输出和STATUS/LAST_ERR轮询机制
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.触发各类错误事件（帧中止、非法opcode、AHB错误等）；
-2.通过RD_CSR(0x11)读STATUS(0x08)和LAST_ERR(0x0C)；
-3.连续发送多条错误命令，每次读取STATUS和LAST_ERR。
-期望结果：
-1.无IRQ信号拉高，MVP不实现独立中断输出；
-2.错误信息通过STATUS和LAST_ERR寄存器查询；
-3.每次错误状态通过响应帧8bit状态码直接返回，前一条错误被新命令覆盖。
-coverage check点：
-对STATUS和LAST_ERR寄存器值的变化收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_015</t>
-  </si>
-  <si>
-    <t>aplc_error_priority_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证前置错误优先级链和单错误返回
-配置条件：
-1.配置clk_i=100MHz，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.4-bit模式下发送WR_CSR帧，pcs_n_i在rx_count&lt;expected_rx_bits时提前拉高(opcode已锁存)→触发STS_FRAME_ERR(0x01)；
-2.test_mode_i=0, en_i=1时发送有效命令→触发STS_NOT_IN_TEST(0x04)；
-3.test_mode_i=1, en_i=0时发送有效命令→触发STS_DISABLED(0x08)；
-4.发送WR_CSR/RD_CSR命令，reg_addr&gt;=0x40→触发STS_BAD_REG(0x10)；
-5.发送AHB_WR32/AHB_RD32命令，addr[1:0]!=2'b00→触发STS_ALIGN_ERR(0x20)。
-期望结果：
-1.各前置错误返回对应状态码，不发起CSR/AHB访问；
-2.优先级链正确：FRAME_ERR(0x01)&gt;BAD_OPCODE(0x02)&gt;NOT_IN_TEST(0x04)&gt;DISABLED(0x08)&gt;BAD_REG(0x10)&gt;ALIGN_ERR(0x20)。
-coverage check点：
-对前置错误的6种类型收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_016</t>
-  </si>
-  <si>
-    <t>aplc_multi_error_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证多错误同时发生时仅返回最高优先级错误
-配置条件：
-1.配置clk_i=100MHz，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.test_mode_i=0, en_i=0时发送非对齐地址的AHB命令（同时满足NOT_IN_TEST+DISABLED+ALIGN_ERR）；
-2.test_mode_i=0, en_i=1时发送reg_addr&gt;=0x40的RD_CSR命令（同时满足NOT_IN_TEST+BAD_REG）；
-3.帧中止+非法opcode组合（发送部分帧后提前拉高pcs_n_i，且opcode非法）。
-期望结果：
-1.按固定优先级链仅报告最高优先级错误，仅返回一个状态码；
-2.任何前置错误均在发起CSR/AHB访问前收敛，不产生副作用。
-coverage check点：
-对多错误组合的优先级仲裁结果收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_017</t>
-  </si>
-  <si>
-    <t>aplc_ahb_error_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证AHB执行期hresp_i=1错误处理
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.AHB从设备配置为返回hresp_i=1。
-输入激励：
-1.发送AHB_WR32(0x20)命令，从设备返回hresp_i=1；
-2.发送AHB_RD32(0x21)命令，从设备返回hresp_i=1；
-3.观测FSM状态恢复。
-期望结果：
-1.STATE_WAIT检测到hresp_i=1后转STATE_ERR；返回STS_AHB_ERR(0x40)；
-2.前置错误与AHB错误互斥，前置检查通过后才可能发生AHB错误；
-3.STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans=IDLE、haddr=0。
-coverage check点：
-对AHB写/读操作返回hresp_i=1的场景收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_018</t>
-  </si>
-  <si>
-    <t>aplc_ahb_timeout_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证AHB超时256周期检测
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.AHB从设备配置为持续返回hready_i=0超过256周期。
-输入激励：
-1.发送AHB_WR32(0x20)命令，hready_i持续为0超过256周期；
-2.发送AHB_RD32(0x21)命令，hready_i持续为0超过256周期；
-3.观测9-bit超时计数器行为。
-期望结果：
-1.9-bit计数器在STATE_WAIT递增，达BUS_TIMEOUT_CYCLES-1(默认255)触发STATE_ERR；
-2.返回STS_AHB_ERR(0x40)；
-3.超时阈值为256周期。
-coverage check点：
-对AHB超时计数器边界值(254/255/256)收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_019</t>
-  </si>
-  <si>
-    <t>aplc_lowpower_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证空闲态低功耗行为
-配置条件：
-1.配置clk_i=100MHz，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.模块空闲态(pcs_n_i=1)下，观测接收/发送移位寄存器和超时计数器；
-2.test_mode_i=0或无有效任务时，观测AHB输出端口；
-3.模块处于STATE_WAIT(AHB等待态)时，观测超时计数器。
-期望结果：
-1.空闲态下接收/发送移位寄存器不更新、不翻转；
-2.htrans_o保持IDLE(2'b00)，无AHB总线翻转；
-3.仅在STATE_WAIT期间超时计数器递增，STATE_REQ时清零，IDLE态不工作。
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_020</t>
-  </si>
-  <si>
-    <t>aplc_latency_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证端到端时延测量
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1；
-2.AHB从设备配置为hready_i=1(零等待)。
-输入激励：
-1.4-bit模式下发送AHB_RD32(0x21)命令，测量端到端延时；
-2.4-bit模式下发送AHB_WR32(0x20)命令，测量端到端延时；
-3.1-bit模式下发送AHB_RD32(0x21)命令，测量端到端延时；
-4.1-bit模式下发送WR_CSR(0x10)命令，测量端到端延时。
-期望结果：
-1.4-bit AHB_RD32: 请求10cyc+译码1~2cyc+AHB 1~N cyc+turnaround 1cyc+响应10cyc ≈ 23~24 cycles最小延时；
-2.4-bit AHB_WR32: 请求18cyc+执行2cyc+turnaround 1cyc+响应2cyc ≈ 23 cycles最小延时；
-3.1-bit AHB_RD32: 请求40cyc+译码1~2cyc+AHB 1~N cyc+turnaround 1cyc+响应40cyc ≈ 83~84 cycles最小延时；
-4.1-bit WR_CSR: 请求48cyc+执行~6cyc+turnaround 1cyc+响应8cyc ≈ 63 cycles最小延时。
-coverage check点：
-对1-bit/4-bit模式与四类opcode的时延组合收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_021</t>
-  </si>
-  <si>
-    <t>aplc_dfx_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证DFX内部调试点可观测性
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.仿真/调试环境。
-输入激励：
-1.运行各类命令（WR_CSR/RD_CSR/AHB_WR32/AHB_RD32），观测内部调试点；
-2.触发各类错误事件，观测错误状态调试点。
-期望结果：
-1.可观测front_state、back_state、opcode、addr、wdata、rdata、status_code、rx_count、tx_count、lane_mode等信号；
-2.便于波形定位和故障复现。
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_022</t>
-  </si>
-  <si>
-    <t>aplc_memmap_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证CSR不进入AHB memory map和AHB地址空间约束
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
-2.SoC集成环境。
-输入激励：
-1.检查模块CSR是否出现在AHB memory map中；
-2.发起AHB_WR32(0x20)/AHB_RD32(0x21)命令访问不同地址。
-期望结果：
-1.模块CSR不进入SoC AHB memory map，仅通过协议命令WR_CSR(0x10)/RD_CSR(0x11)访问；
-2.AHB Master采用32bit地址空间和word(32-bit)访问粒度，haddr_o必须4-byte对齐。
-coverage check点：
-对AHB访问地址范围和4-byte对齐约束收集功能覆盖率</t>
-  </si>
-  <si>
-    <t>TC_023</t>
-  </si>
-  <si>
-    <t>aplc_ahb_2phase_test</t>
-  </si>
-  <si>
-    <t>TC场景：验证AHB-Lite 2-phase流水时序、固定属性和错误恢复
-配置条件：
-1.配置clk_i=100MHz，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)。
-输入激励：
-1.发送AHB_WR32(0x20)命令，观测AHB 2-phase写流水时序（haddr_o/hwrite_o/htrans_o/hwdata_o）；
-2.发送AHB_RD32(0x21)命令，观测AHB 2-phase读流水时序（haddr_o/htrans_o/hrdata_i/hready_i）；
-3.检查hsize_o和hburst_o输出；
-4.观测htrans_o在不同FSM状态下的值；
-5.触发AHB错误(STATE_ERR)后观测FSM状态恢复。
-期望结果：
-1.T1(STATE_REQ)驱动haddr_o/hwrite_o=1/htrans_o=NONSEQ(2'b10)；T2(STATE_WAIT)htrans_o回到IDLE(2'b00)，写驱动hwdata_o，读在hready_i=1时采样hrdata_i；haddr与hwdata错开1拍；
-2.hsize_o固定输出3'b010(WORD)，hburst_o固定输出3'b000(SINGLE)；
-3.htrans_o仅在STATE_REQ驱动NONSEQ(2'b10)持续1周期，其余时刻均为IDLE(2'b00)；
-4.STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans=IDLE、haddr=0。
-coverage check点：
-对AHB写/读2-phase流水时序和htrans_o状态收集功能覆盖率</t>
+1. 收集空闲态下各寄存器翻转率的覆盖率
+2. 收集AHB输出在非工作模式下的状态覆盖率</t>
   </si>
   <si>
     <t>Feature List分解表格</t>
@@ -883,6 +890,9 @@
 期望：前置检查检测到en_i=0，返回STS_DISABLED(0x08)，不发起CSR/AHB访问。</t>
   </si>
   <si>
+    <t>CHK_007</t>
+  </si>
+  <si>
     <t>TP_011</t>
   </si>
   <si>
@@ -891,6 +901,9 @@
 期望：前置检查通过，正常执行命令并返回正确状态码和数据。</t>
   </si>
   <si>
+    <t>CHK_006, CHK_007</t>
+  </si>
+  <si>
     <t>TP_012</t>
   </si>
   <si>
@@ -899,6 +912,9 @@
 期望：每拍收发1bit(pdi_i[0])；帧接收周期为帧长bit数；命令执行正确。</t>
   </si>
   <si>
+    <t>CHK_008</t>
+  </si>
+  <si>
     <t>TP_013</t>
   </si>
   <si>
@@ -915,7 +931,7 @@
 期望：pcs_n_i=1时空闲；pcs_n_i=0时开启帧接收；pcs_n_i拉高时结束事务。</t>
   </si>
   <si>
-    <t>CHK_007</t>
+    <t>CHK_009, CHK_011</t>
   </si>
   <si>
     <t>TP_015</t>
@@ -926,6 +942,9 @@
 期望：1-bit模式仅bit0有效，其余位忽略；4-bit模式全部4位有效；MSB-first顺序传输。</t>
   </si>
   <si>
+    <t>CHK_008, CHK_009</t>
+  </si>
+  <si>
     <t>TP_016</t>
   </si>
   <si>
@@ -934,6 +953,9 @@
 期望：响应阶段pdo_oe_o=1，模块驱动pdo_o输出数据；非发送阶段pdo_oe_o=0，pdo_o值无意义；半双工，主机和模块不同时驱动。</t>
   </si>
   <si>
+    <t>CHK_009, CHK_010</t>
+  </si>
+  <si>
     <t>TP_017</t>
   </si>
   <si>
@@ -942,6 +964,9 @@
 期望：接收48bit(opcode8+reg_addr8+wdata32)后产生frame_valid；响应8bit状态码。</t>
   </si>
   <si>
+    <t>CHK_009</t>
+  </si>
+  <si>
     <t>TP_018</t>
   </si>
   <si>
@@ -974,6 +999,9 @@
 期望：产生frame_abort；返回STS_FRAME_ERR(0x01)；不发起CSR/AHB访问。</t>
   </si>
   <si>
+    <t>CHK_011</t>
+  </si>
+  <si>
     <t>TP_022</t>
   </si>
   <si>
@@ -982,6 +1010,9 @@
 期望：请求阶段与响应阶段之间固定插入1个clk_i周期turnaround；turnaround期间pdo_oe_o=0；TX阶段pdo_oe_o=1。</t>
   </si>
   <si>
+    <t>CHK_010</t>
+  </si>
+  <si>
     <t>TP_023</t>
   </si>
   <si>
@@ -990,7 +1021,7 @@
 期望：前端收满8bit后锁存opcode；根据opcode确定expected_rx_bits；正确发起对应类型任务。</t>
   </si>
   <si>
-    <t>CHK_008</t>
+    <t>CHK_012</t>
   </si>
   <si>
     <t>TP_024</t>
@@ -1009,7 +1040,7 @@
 期望：LANE_MODE=00对应1-bit模式，01对应4-bit模式；SOFT_RST写1触发协议上下文清零并恢复默认lane模式。</t>
   </si>
   <si>
-    <t>CHK_009</t>
+    <t>CHK_003, CHK_004</t>
   </si>
   <si>
     <t>TP_026</t>
@@ -1036,7 +1067,7 @@
 期望：MVP版本不实现独立中断输出；无IRQ信号拉高；错误信息通过STATUS寄存器和LAST_ERR寄存器查询。</t>
   </si>
   <si>
-    <t>CHK_010</t>
+    <t>CHK_006, CHK_007, CHK_014</t>
   </si>
   <si>
     <t>TP_029</t>
@@ -1055,9 +1086,6 @@
 期望：产生frame_abort，返回STS_FRAME_ERR(0x01)，不发起CSR/AHB访问。</t>
   </si>
   <si>
-    <t>CHK_011</t>
-  </si>
-  <si>
     <t>TP_031</t>
   </si>
   <si>
@@ -1098,7 +1126,7 @@
 期望：返回STS_ALIGN_ERR(0x20)，不发起AHB访问。</t>
   </si>
   <si>
-    <t>CHK_012</t>
+    <t>CHK_013</t>
   </si>
   <si>
     <t>TP_036</t>
@@ -1109,7 +1137,7 @@
 期望：STATE_WAIT检测到hresp_i=1，转STATE_ERR；返回STS_AHB_ERR(0x40)。</t>
   </si>
   <si>
-    <t>CHK_013</t>
+    <t>CHK_015</t>
   </si>
   <si>
     <t>TP_037</t>
@@ -1128,6 +1156,9 @@
 期望：按固定优先级链仅报告最高优先级错误：FRAME_ERR(0x01)&gt;BAD_OPCODE(0x02)&gt;NOT_IN_TEST(0x04)&gt;DISABLED(0x08)&gt;BAD_REG(0x10)&gt;ALIGN_ERR(0x20)；仅返回一个状态码。</t>
   </si>
   <si>
+    <t>CHK_014</t>
+  </si>
+  <si>
     <t>TP_039</t>
   </si>
   <si>
@@ -1144,7 +1175,7 @@
 期望：接收移位寄存器不更新；发送移位寄存器不翻转；超时计数器不工作。</t>
   </si>
   <si>
-    <t>CHK_014</t>
+    <t>CHK_019</t>
   </si>
   <si>
     <t>TP_041</t>
@@ -1171,7 +1202,7 @@
 期望：请求接收10cyc + 译码1~2cyc + AHB返回1~N cyc + turnaround 1cyc + 响应发送10cyc ≈ 23~24 cycles最小延时。</t>
   </si>
   <si>
-    <t>CHK_015</t>
+    <t>CHK_016</t>
   </si>
   <si>
     <t>TP_044</t>
@@ -1211,7 +1242,7 @@
 期望：可观测front_state、back_state、opcode、addr、wdata、rdata、status_code、rx_count、tx_count、lane_mode等信号；便于波形定位和故障复现。</t>
   </si>
   <si>
-    <t>CHK_016</t>
+    <t>CHK_020</t>
   </si>
   <si>
     <t>TP_049</t>
@@ -1222,7 +1253,7 @@
 期望：模块CSR不进入SoC AHB memory map，仅通过协议命令(WR_CSR/RD_CSR)访问。</t>
   </si>
   <si>
-    <t>CHK_017</t>
+    <t>CHK_021</t>
   </si>
   <si>
     <t>TP_050</t>
@@ -1257,12 +1288,18 @@
 期望：hsize_o固定输出3'b010(WORD)；hburst_o固定输出3'b000(SINGLE)；不支持byte/halfword与burst传输。</t>
   </si>
   <si>
+    <t>CHK_018</t>
+  </si>
+  <si>
     <t>TP_054</t>
   </si>
   <si>
     <t>条件：AHB命令执行期间。
 激励：观测htrans_o在不同FSM状态下的值。
 期望：htrans_o仅在STATE_REQ(地址相)驱动NONSEQ(2'b10)持续1周期；其余时刻均为IDLE(2'b00)。</t>
+  </si>
+  <si>
+    <t>CHK_017</t>
   </si>
   <si>
     <t>TP_055</t>
@@ -1310,177 +1347,236 @@
     <t>CHK描述</t>
   </si>
   <si>
-    <t>clk_freq_checker</t>
-  </si>
-  <si>
-    <t>对于时钟，检查clk_i频率稳定性和目标频率约束：
-1、频率值检查：连续采集clk_i上升沿和下降沿，计算实际周期，判断是否处于100MHz目标频率的允许误差范围内（±1%）；
-2、时钟稳定性检查：通过连续采样clk_i周期，对比相邻两个周期的频率偏差是否在3%内；
-3、单时钟域验证：确认协议接收（pdi_i采样）、状态机控制（front_state/back_state跳转）和AHB-Lite主接口（haddr_o/htrans_o驱动）均在clk_i上升沿同步，无跨时钟域问题。</t>
-  </si>
-  <si>
-    <t>reset_checker</t>
-  </si>
-  <si>
-    <t>对于复位，检查rst_n_i异步复位与同步释放行为及复位后状态：
-1、异步复位触发检查：rst_n_i下降沿立即触发复位，无需等待clk_i上升沿；
-2、同步释放检查：rst_n_i释放时在clk_i上升沿同步退出复位；
-3、FSM状态恢复检查：复位后front_state=IDLE(3'd0)，back_state=S_IDLE(3'd0)；
-4、输出默认值检查：复位后pdo_oe_o=0，htrans_o=2'b00(IDLE)，csr_rd_en_o=0，csr_wr_en_o=0，pdo_o=4'b0；
-5、寄存器默认值检查：CTRL.EN=0，CTRL.LANE_MODE=2'b00(1-bit默认模式)，所有协议/响应上下文清空，错误状态清除。</t>
-  </si>
-  <si>
-    <t>csr_write_checker</t>
-  </si>
-  <si>
-    <t>对于CSR写操作，检查WR_CSR(0x10)命令的写时序和数据正确性：
-1、写使能脉冲检查：csr_wr_en_o脉冲持续1个clk_i周期，同周期csr_addr_o和csr_wdata_o有效；
-2、地址范围检查：csr_addr_o有效范围为0x00~0x3F，对应VERSION(0x00)、CTRL(0x04)、STATUS(0x08)、LAST_ERR(0x0C)；
-3、写数据检查：外部CSR File在csr_wr_en_o=1的同周期采样csr_addr_o/csr_wdata_o并写入；
-4、响应检查：写操作完成后返回STS_OK(0x00)状态码。</t>
-  </si>
-  <si>
-    <t>csr_read_checker</t>
-  </si>
-  <si>
-    <t>对于CSR读操作，检查RD_CSR(0x11)命令的读时序和数据正确性：
-1、读使能脉冲检查：csr_rd_en_o脉冲持续1个clk_i周期；
-2、1周期读延迟检查：外部CSR File在csr_rd_en_o脉冲后的下一个clk_i周期将读数据稳定在csr_rdata_i[31:0]上；
-3、读数据正确性检查：模块正确采样csr_rdata_i，响应帧中RDATA[31:0]与CSR File返回值一致；
-4、响应检查：读操作完成后返回STS_OK(0x00)+RDATA[31:0]。</t>
-  </si>
-  <si>
-    <t>csr_bad_reg_checker</t>
-  </si>
-  <si>
-    <t>对于CSR非法地址检测，检查reg_addr&gt;=0x40时的前置拒绝行为：
-1、非法地址检测检查：当WR_CSR(0x10)或RD_CSR(0x11)命令的reg_addr&gt;=0x40(CSR_ADDR_MAX=0x3F)时，前置检查拒绝访问；
-2、状态码检查：返回STS_BAD_REG(0x10)；
-3、不发起访问检查：csr_rd_en_o=0，csr_wr_en_o=0，不发起CSR读/写操作。</t>
-  </si>
-  <si>
-    <t>mode_gate_checker</t>
-  </si>
-  <si>
-    <t>对于工作模式，检查test_mode_i和en_i的前置门控以及lane模式切换：
-1、test_mode_i门控检查：test_mode_i=0时，任何命令均返回STS_NOT_IN_TEST(0x04)，不发起CSR/AHB访问；
-2、en_i门控检查：test_mode_i=1且en_i=0时，任何命令均返回STS_DISABLED(0x08)，不发起CSR/AHB访问；
-3、正常模式检查：test_mode_i=1且en_i=1时，前置检查通过，正常执行命令并返回正确状态码和数据；
-4、1-bit模式检查：lane_mode_i=2'b00时，每拍仅pdi_i[0]有效，帧接收周期为帧长bit数；
-5、4-bit模式检查：lane_mode_i=2'b01时，每拍pdi_i[3:0]均有效，帧接收周期为帧长/4。</t>
-  </si>
-  <si>
-    <t>frame_io_checker</t>
-  </si>
-  <si>
-    <t>对于数据接口，检查类SPI帧协议的时序和数据正确性：
-1、帧边界检查：pcs_n_i=1时模块空闲；pcs_n_i拉低时开启帧接收；pcs_n_i拉高时结束事务；
-2、输入数据检查：1-bit模式仅pdi_i[0]有效；4-bit模式pdi_i[3:0]均有效；所有数据MSB-first顺序传输；
-3、输出方向检查：响应阶段pdo_oe_o=1，模块驱动pdo_o[3:0]输出数据；非发送阶段pdo_oe_o=0，pdo_o值无意义；
-4、帧长度检查：WR_CSR(0x10)接收48bit(opcode8+reg_addr8+wdata32)；RD_CSR(0x11)接收16bit(opcode8+reg_addr8)；AHB_WR32(0x20)接收72bit(opcode8+addr32+wdata32)；AHB_RD32(0x21)接收40bit(opcode8+addr32)；
-5、响应格式检查：写类命令响应8bit状态码；读类命令响应40bit(8bit状态+32bit读数据)；
-6、帧中止检查：帧接收未完成时pcs_n_i提前拉高，产生frame_abort，返回STS_FRAME_ERR(0x01)，不发起CSR/AHB访问；
-7、turnaround检查：请求阶段与响应阶段之间固定插入1个clk_i周期turnaround；turnaround期间pdo_oe_o=0；TX阶段pdo_oe_o=1。</t>
+    <t>clk_i_freq_checker</t>
+  </si>
+  <si>
+    <t>检查clk_i时钟频率和稳定性：
+1. 连续采集clk_i上升沿和下降沿，计算实际频率/周期，判断是否处于100MHz目标频率的允许误差范围内（±1%）
+2. 检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内
+3. 检查所有内部逻辑在clk_i上升沿正确同步，无跨时钟域问题
+4. 检查AHB-Lite主接口与协议侧共用clk_i，同域工作</t>
+  </si>
+  <si>
+    <t>rst_ni_reset_checker</t>
+  </si>
+  <si>
+    <t>检查rst_ni异步复位与同步释放行为：
+1. rst_ni下降沿立即触发复位，无需等待clk_i上升沿（异步有效）
+2. rst_ni上升沿释放时，在下一个clk_i上升沿同步退出复位状态
+3. 复位后检查所有输出deassert：pdo_oe_o=0, htrans_o=2'b00(IDLE), csr_rd_en_o=0, csr_wr_en_o=0, pdo_o=4'b0
+4. 复位后检查前端FSM状态front_state=IDLE(3'd0)，后端FSM状态back_state=S_IDLE(3'd0)
+5. 复位后检查所有协议/响应上下文清空，错误状态清除
+6. 检查复位不改变en_i、lane_mode_i、test_mode_i等外部输入端口（由集成方控制）</t>
+  </si>
+  <si>
+    <t>csr_write_timing_checker</t>
+  </si>
+  <si>
+    <t>检查CSR写操作时序正确性：
+1. csr_wr_en_o脉冲持续1个clk_i周期
+2. 同周期csr_addr_o和csr_wdata_o有效：外部CSR File在该周期采样csr_addr_o和csr_wdata_o完成写入
+3. CSR写操作始终返回STS_OK(0x00)
+4. 写命令响应帧长度为8bit（仅status byte）
+5. 检查CSR有效地址范围0x00~0x3F内的访问正常发起csr_wr_en_o</t>
+  </si>
+  <si>
+    <t>csr_read_timing_checker</t>
+  </si>
+  <si>
+    <t>检查CSR读操作时序正确性：
+1. csr_rd_en_o脉冲持续1个clk_i周期
+2. 外部CSR File在csr_rd_en_o脉冲后的下一个clk_i周期将读数据稳定在csr_rdata_i[31:0]上（1 cycle读延迟）
+3. 模块在该周期正确采样csr_rdata_i
+4. CSR读操作返回STS_OK(0x00)+rdata[31:0]
+5. 读命令响应帧长度为40bit（8bit status + 32bit rdata），MSB-first</t>
+  </si>
+  <si>
+    <t>csr_addr_range_checker</t>
+  </si>
+  <si>
+    <t>检查CSR地址范围约束：
+1. CSR有效地址范围为0x00~0x3F（reg_addr &lt; 0x40）
+2. reg_addr&gt;=0x40的请求在前置检查阶段即被拒绝，返回STS_BAD_REG(0x10)
+3. 不发起CSR读/写操作：csr_rd_en_o=0, csr_wr_en_o=0
+4. csr_addr_o[7:0]仅驱动0x00~0x3F范围内的地址，不出现&gt;=0x40的值</t>
+  </si>
+  <si>
+    <t>test_mode_checker</t>
+  </si>
+  <si>
+    <t>检查test_mode_i前置条件：
+1. SLC_DPCHK在frame_valid时刻组合采样test_mode_i
+2. test_mode_i=0时，所有命令被前置检查拒绝，返回STS_NOT_IN_TEST(0x04)
+3. 不发起任何CSR/AHB访问：csr_rd_en_o=0, csr_wr_en_o=0, htrans_o=IDLE(2'b00)
+4. 模块在协议层仍正常工作（接收帧→返回错误状态码），但无总线事务
+5. 帧接收期间test_mode_i不影响SLC_CAXIS接收过程</t>
+  </si>
+  <si>
+    <t>en_checker</t>
+  </si>
+  <si>
+    <t>检查en_i模块使能前置条件：
+1. en_i=0时，所有命令被前置检查拒绝，返回STS_DISABLED(0x08)
+2. 不发起任何CSR/AHB访问：csr_rd_en_o=0, csr_wr_en_o=0, htrans_o=IDLE(2'b00)
+3. en_i由SoC集成方硬件端口提供，非CSR可配
+4. en_i在frame_valid时刻被前置检查采样
+5. test_mode_i=1且en_i=0时，优先级：STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08)</t>
+  </si>
+  <si>
+    <t>lane_mode_checker</t>
+  </si>
+  <si>
+    <t>检查lane_mode_i通道模式配置正确性：
+1. lane_mode_i=2'b00时，1-bit模式：每拍收发1bit，仅使用pdi_i[0]/pdo_o[0]，其余位忽略
+2. lane_mode_i=2'b01时，4-bit模式：每拍收发4bit，使用pdi_i[3:0]/pdo_o[3:0]
+3. 接收器(SLC_CAXIS)和发送器(SLC_SAXIS)连续组合采样lane_mode_i，计算bpc(bits per clock)
+4. 1-bit模式bpc=1，4-bit模式bpc=4
+5. 数据按MSB-first顺序传输，4-bit模式按高nibble优先发送</t>
+  </si>
+  <si>
+    <t>frame_format_checker</t>
+  </si>
+  <si>
+    <t>检查帧格式和帧长正确性：
+1. WR_CSR(0x10)：帧结构[opcode(8)|reg_addr(8)|wdata(32)]=48bit，接收后产生frame_valid，响应8bit状态码
+2. RD_CSR(0x11)：帧结构[opcode(8)|reg_addr(8)]=16bit，接收后产生frame_valid，响应40bit(status8+rdata32)
+3. AHB_WR32(0x20)：帧结构[opcode(8)|addr(32)|wdata(32)]=72bit，接收后产生frame_valid，响应8bit状态码
+4. AHB_RD32(0x21)：帧结构[opcode(8)|addr(32)]=40bit，接收后产生frame_valid，响应40bit(status8+rdata32)
+5. 接收器使用80-bit移位寄存器rx_shift_q，前8bit完成后锁存opcode确定expected_rx_bits
+6. next_count&gt;=expected_rx_bits时产生frame_valid（寄存输出，延迟1 cycle）</t>
+  </si>
+  <si>
+    <t>turnaround_checker</t>
+  </si>
+  <si>
+    <t>检查请求-响应之间的turnaround时序：
+1. 请求阶段与响应阶段之间固定插入1个clk_i周期的turnaround
+2. turnaround期间pdo_oe_o=0（SAXIS在TA态不驱动pdo_o）
+3. TX阶段开始时pdo_oe_o=1，SAXIS加载移位寄存器开始移位输出
+4. 前端FSM从WAIT_RESP进入TA(3'd4)状态持续1个clk_i周期，再进入TX(3'd5)状态
+5. resp_valid有效后锁存status/rdata，tx_start启动SAXIS发送</t>
+  </si>
+  <si>
+    <t>frame_abort_checker</t>
+  </si>
+  <si>
+    <t>检查帧中止(frame_abort)检测和响应：
+1. pcs_n_i在rx_count&lt;expected_rx_bits时提前拉高（且opcode已锁存），产生frame_abort（寄存输出，延迟1 cycle）
+2. pcs_n_i在opcode锁存前（接收不足8bit）即拉高：接收状态静默复位，不产生frame_abort，不返回任何状态码
+3. frame_abort产生后：不发起CSR/AHB访问，返回STS_FRAME_ERR(0x01)
+4. 前端FSM走IDLE→TA→TX错误返回路径（跳过ISSUE/WAIT_RESP）
+5. pcs_n_i在TX阶段拉高：前端FSM直接回到IDLE，当前响应截断，不产生新错误码</t>
   </si>
   <si>
     <t>opcode_checker</t>
   </si>
   <si>
-    <t>对于opcode解析，检查合法与非法opcode的处理：
-1、合法opcode检查：前端收满8bit后锁存opcode，根据opcode确定expected_rx_bits——0x10(WR_CSR)对应48bit、0x11(RD_CSR)对应16bit、0x20(AHB_WR32)对应72bit、0x21(AHB_RD32)对应40bit；正确发起对应类型任务；
-2、非法opcode检查：opcode不在{0x10,0x11,0x20,0x21}中时，前置检查返回STS_BAD_OPCODE(0x02)，不发起CSR/AHB访问。</t>
-  </si>
-  <si>
-    <t>ctrl_reg_checker</t>
-  </si>
-  <si>
-    <t>对于CTRL寄存器配置，检查EN/LANE_MODE/SOFT_RST字段功能：
-1、EN字段检查：CTRL.EN=1时模块使能，CTRL.EN=0时返回STS_DISABLED(0x08)；
-2、LANE_MODE字段检查：CTRL.LANE_MODE=2'b00对应1-bit模式，2'b01对应4-bit模式，其他值为非法（MVP不支持）；
-3、SOFT_RST字段检查：CTRL.SOFT_RST写1触发协议上下文清零并恢复默认lane模式（1-bit）；
-4、事务期间lane切换检查：pcs_n_i=0(事务执行期间)lane_mode_i变化时，移位宽度bpc立即改变，帧数据错位，模块不检测此违规，可能误触发STS_BAD_OPCODE(0x02)或STS_FRAME_ERR(0x01)；
-5、空闲态lane切换检查：pcs_n_i=1(空闲态)切换lane_mode_i后，新事务使用更新后的lane模式，帧数据正确。</t>
-  </si>
-  <si>
-    <t>status_polling_checker</t>
-  </si>
-  <si>
-    <t>对于中断与状态查询，检查MVP无中断输出和轮询机制：
-1、无中断输出检查：MVP版本不实现独立中断输出，无IRQ信号拉高；
-2、STATUS寄存器检查：错误与完成状态通过STATUS寄存器查询，busy指示正确；
-3、LAST_ERR寄存器检查：最近错误类型通过LAST_ERR寄存器查询，值与状态码对应；
-4、轮询覆盖检查：连续发送多条错误命令时，每次错误状态通过响应帧8bit状态码直接返回给ATE，前一条错误信息被新命令覆盖。</t>
+    <t>检查opcode解码和合法性：
+1. 有效opcode集合：{0x10(WR_CSR), 0x11(RD_CSR), 0x20(AHB_WR32), 0x21(AHB_RD32)}
+2. 前端收满8bit后锁存opcode，根据opcode确定expected_rx_bits
+3. opcode不在有效集合中时，前置检查返回STS_BAD_OPCODE(0x02)，不发起CSR/AHB访问
+4. 接收完成后模块执行左归一化（left-normalization），opcode始终位于rx_data[79:72]
+5. 非法opcode优先级：FRAME_ERR(0x01) &gt; STS_BAD_OPCODE(0x02)</t>
+  </si>
+  <si>
+    <t>align_err_checker</t>
+  </si>
+  <si>
+    <t>检查AHB地址对齐约束：
+1. AHB地址必须4-byte对齐：addr[1:0]=2'b00
+2. addr[1:0]!=2'b00时，前置检查返回STS_ALIGN_ERR(0x20)，不发起AHB访问
+3. 不驱动htrans_o=NONSEQ，不驱动haddr_o
+4. STS_ALIGN_ERR(0x20)优先级最低，仅当所有更高级别前置检查通过后才可能报告</t>
   </si>
   <si>
     <t>error_priority_checker</t>
   </si>
   <si>
-    <t>对于前置错误优先级，检查固定优先级链和多错误同时发生时的行为：
-1、优先级链检查：前置检查按固定优先级返回错误——STS_FRAME_ERR(0x01) &gt; STS_BAD_OPCODE(0x02) &gt; STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08) &gt; STS_BAD_REG(0x10) &gt; STS_ALIGN_ERR(0x20)；
-2、多错误场景检查：同时满足多个前置错误条件时，仅报告最高优先级错误，仅返回一个状态码；
-3、前置收敛检查：任何前置错误均在发起CSR/AHB访问前收敛，不产生副作用。</t>
-  </si>
-  <si>
-    <t>ahb_align_checker</t>
-  </si>
-  <si>
-    <t>对于AHB地址对齐，检查addr[1:0]!=2'b00时的前置拒绝行为：
-1、对齐检测检查：AHB_WR32(0x20)或AHB_RD32(0x21)命令的addr[1:0]!=2'b00时，前置检查拒绝访问；
-2、状态码检查：返回STS_ALIGN_ERR(0x20)；
-3、不发起AHB访问检查：htrans_o保持IDLE(2'b00)，不发起AHB总线事务。</t>
+    <t>检查多错误并发时的优先级链：
+1. 前置检查按固定优先级链（if-else链实现）仅报告最高优先级错误：
+   STS_FRAME_ERR(0x01) &gt; STS_BAD_OPCODE(0x02) &gt; STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08) &gt; STS_BAD_REG(0x10) &gt; STS_ALIGN_ERR(0x20)
+2. 不存在多错误同时上报的情况，每次仅报告一个状态码
+3. STS_AHB_ERR(0x40)不在优先级链中——AHB错误仅在所有前置检查通过后才可能发生，与前置错误互斥
+4. SLC_DPCHK对frame_valid/frame_abort/opcode/test_mode_i/en_i/reg_addr/addr进行组合逻辑检查
+5. 输出chk_err_code和chk_pass信号</t>
   </si>
   <si>
     <t>ahb_error_checker</t>
   </si>
   <si>
-    <t>对于AHB执行期错误，检查hresp_i错误和超时两种情况：
-1、hresp_i错误检查：AHB从设备返回hresp_i=1时，STATE_WAIT检测到后转STATE_ERR，返回STS_AHB_ERR(0x40)；
-2、超时检查：9-bit计数器在STATE_WAIT每拍+1，达BUS_TIMEOUT_CYCLES-1(默认255)触发STATE_ERR，返回STS_AHB_ERR(0x40)；
-3、超时计数器复位检查：STATE_REQ时计数器清零；
-4、AHB错误与前置错误互斥检查：前置检查通过后才可能发生AHB错误，STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans=IDLE、haddr=0。</t>
-  </si>
-  <si>
-    <t>lowpower_checker</t>
-  </si>
-  <si>
-    <t>对于低功耗，检查空闲态下寄存器/计数器不更新和AHB输出保持IDLE：
-1、移位寄存器检查：空闲态(pcs_n_i=1)下接收/发送移位寄存器不更新、不翻转；
-2、AHB输出检查：test_mode_i=0或无有效任务时，htrans_o保持IDLE(2'b00)，无AHB总线翻转；
-3、超时计数器检查：仅在STATE_WAIT期间超时计数器递增，STATE_REQ时清零，IDLE态不工作。</t>
-  </si>
-  <si>
-    <t>latency_checker</t>
-  </si>
-  <si>
-    <t>对于性能时延，检查端到端延时和超时阈值：
-1、4-bit AHB_RD32时延检查：请求接收10cyc + 译码1~2cyc + AHB返回1~N cyc + turnaround 1cyc + 响应发送10cyc ≈ 23~24 cycles最小延时；
-2、4-bit AHB_WR32时延检查：请求接收18cyc + 执行2cyc + turnaround 1cyc + 响应发送2cyc ≈ 23 cycles最小延时；
-3、1-bit AHB_RD32时延检查：请求接收40cyc + 译码1~2cyc + AHB返回1~N cyc + turnaround 1cyc + 响应发送40cyc ≈ 83~84 cycles最小延时；
-4、1-bit WR_CSR时延检查：请求接收48cyc + 执行~6cyc + turnaround 1cyc + 响应发送8cyc ≈ 63 cycles最小延时；
-5、超时阈值检查：9-bit计数器在STATE_WAIT递增，达BUS_TIMEOUT_CYCLES-1(默认255)触发STATE_ERR，超时阈值为256周期。</t>
-  </si>
-  <si>
-    <t>dfx_checker</t>
-  </si>
-  <si>
-    <t>对于DFX可观测性，检查内部调试点信号是否可观测：
-1、FSM状态可观测检查：front_state和back_state可被外部观测；
-2、协议字段可观测检查：opcode、addr、wdata、rdata、status_code可被外部读取；
-3、计数器可观测检查：rx_count和tx_count可被外部读取；
-4、配置可观测检查：lane_mode信号可被外部观测。</t>
-  </si>
-  <si>
-    <t>ahb_proto_checker</t>
-  </si>
-  <si>
-    <t>对于AHB-Lite协议，检查2-phase流水时序、固定属性和错误恢复：
-1、2-phase写时序检查：T1(STATE_REQ)驱动haddr_o/hwrite_o=1/htrans_o=NONSEQ(2'b10)；T2(STATE_WAIT)htrans_o回到IDLE(2'b00)，驱动hwdata_o；haddr_o与hwdata_o错开1拍；
-2、2-phase读时序检查：T1(STATE_REQ)驱动haddr_o/htrans_o=NONSEQ(2'b10)；T2(STATE_WAIT)htrans_o=IDLE(2'b00)，hready_i=1时采样hrdata_i；
-3、固定属性检查：hsize_o固定输出3'b010(WORD)，hburst_o固定输出3'b000(SINGLE)；
-4、htrans_o状态检查：仅在STATE_REQ(地址相)驱动NONSEQ(2'b10)持续1周期，其余时刻均为IDLE(2'b00)；
-5、错误恢复检查：STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans=IDLE、haddr=0，模块可立即接受新请求；
-6、CSR访问方式检查：模块CSR不进入SoC AHB memory map，仅通过协议命令WR_CSR(0x10)/RD_CSR(0x11)访问；
-7、AHB地址空间检查：AHB Master采用32bit地址空间和word(32-bit)访问粒度，haddr_o必须4-byte对齐。</t>
+    <t>检查AHB总线异常和超时：
+1. AHB错误响应：STATE_WAIT检测到hresp_i=1，转STATE_ERR(3'b100)，返回STS_AHB_ERR(0x40)
+2. AHB超时：9-bit超时计数器timeout_cnt_q在STATE_WAIT每拍递增，STATE_REQ时清零；达BUS_TIMEOUT_CYCLES-1(默认255)触发STATE_ERR
+3. hresp_i=1和超时使用同一状态码STS_AHB_ERR(0x40)，不做区分
+4. STATE_ERR下一拍自动转STATE_IDLE，AHB输出恢复htrans_o=IDLE(2'b00), haddr_o=0
+5. 模块可立即接受新请求，无需外部干预</t>
+  </si>
+  <si>
+    <t>ahb_2phase_checker</t>
+  </si>
+  <si>
+    <t>检查AHB-Lite 2-phase流水时序正确性：
+1. 写操作：T1(STATE_REQ)驱动haddr_o/hwrite_o/htrans_o=NONSEQ(2'b10)；T2(STATE_WAIT)htrans_o回到IDLE(2'b00)，驱动hwdata_o；haddr与hwdata错开1拍
+2. 读操作：T1(STATE_REQ)驱动haddr_o/htrans_o=NONSEQ；T2(STATE_WAIT)htrans_o=IDLE，hready_i=1时采样hrdata_i[31:0]
+3. hsize_o固定输出3'b010(WORD/32-bit)
+4. hburst_o固定输出3'b000(SINGLE)
+5. 不支持byte/halfword与Burst传输</t>
+  </si>
+  <si>
+    <t>ahb_htrans_checker</t>
+  </si>
+  <si>
+    <t>检查AHB htrans_o传输类型信号：
+1. htrans_o仅在STATE_REQ(地址相)驱动NONSEQ(2'b10)，持续1个clk_i周期
+2. 其余时刻htrans_o均为IDLE(2'b00)
+3. 当前事务完成前，不得发起下一笔AHB请求
+4. AHB Master FSM 5态状态转移正确：STATE_IDLE→STATE_REQ→STATE_WAIT→STATE_DONE/STATE_ERR→STATE_IDLE</t>
+  </si>
+  <si>
+    <t>ahb_fixed_signal_checker</t>
+  </si>
+  <si>
+    <t>检查AHB固定输出信号：
+1. hsize_o固定输出3'b010（32-bit/WORD）
+2. hburst_o固定输出3'b000（SINGLE）
+3. 不支持byte/halfword与Burst传输
+4. 仅使用htrans_o的IDLE(2'b00)和NONSEQ(2'b10)两种值
+5. 写数据hwdata_o在STATE_REQ和STATE_WAIT均被驱动以保证稳定性，但从机采样点是数据相(T2)</t>
+  </si>
+  <si>
+    <t>low_power_checker</t>
+  </si>
+  <si>
+    <t>检查空闲态低功耗行为：
+1. pcs_n_i=1(空闲态)时，接收移位寄存器(rx_shift_q)不更新
+2. 非发送阶段(TX/TA态外)，发送移位寄存器不翻转
+3. 超时计数器仅在STATE_WAIT期间递增；STATE_REQ时清零；IDLE态不工作
+4. test_mode_i=0或无有效任务时，htrans_o保持IDLE(2'b00)，无AHB总线翻转
+5. 仅在RX/TX/WAIT_AHB相关状态翻转关键寄存器</t>
+  </si>
+  <si>
+    <t>dfx_observability_checker</t>
+  </si>
+  <si>
+    <t>检查内部调试信号可观测性：
+1. front_state(前端FSM状态)可观测：IDLE(3'd0)/ISSUE(3'd2)/WAIT_RESP(3'd3)/TA(3'd4)/TX(3'd5)
+2. back_state(后端FSM状态)可观测：S_IDLE(3'd0)/S_LOAD_TASK(3'd1)/S_EXEC(3'd2)/S_WAIT_AHB(3'd3)/S_BUILD_RESP(3'd4)/S_DONE(3'd5)
+3. opcode可观测：读取当前命令的操作码
+4. addr/wdata/rdata可观测：地址和读写数据通路
+5. status_code可观测：当前事务的状态码
+6. rx_count/tx_count可观测：接收和发送计数器值
+7. lane_mode可观测：当前通道模式配置</t>
+  </si>
+  <si>
+    <t>memory_map_checker</t>
+  </si>
+  <si>
+    <t>检查CSR地址空间与AHB memory map的独立性：
+1. 模块CSR不进入SoC AHB memory map，仅通过协议命令(WR_CSR/RD_CSR)访问
+2. CSR寄存器访问路径：协议命令→csr_rd_en_o/csr_wr_en_o→外部CSR File
+3. AHB Master访问路径：协议命令→haddr_o/htrans_o→AHB总线
+4. 两种访问路径独立，CSR寄存器不存在于AHB地址空间中
+5. AHB Master采用32bit地址空间和word(32-bit)访问粒度</t>
   </si>
   <si>
     <t>填写要求</t>
@@ -1498,7 +1594,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1510,6 +1606,7 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1517,6 +1614,7 @@
       <sz val="6"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1525,24 +1623,22 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1565,7 +1661,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1660,28 +1756,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1722,9 +1803,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1745,14 +1823,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2040,301 +2118,301 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="17"/>
+      <c r="A1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>95</v>
-      </c>
       <c r="E6" s="9" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="108" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="148.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="67.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="108" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.15">
@@ -2345,68 +2423,68 @@
       <c r="E21"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="22"/>
+      <c r="A22" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="21"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="17"/>
+        <v>60</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="16"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="17"/>
+        <v>61</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="16"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="17"/>
+        <v>62</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="17"/>
+        <v>63</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="17"/>
+        <v>64</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -2563,50 +2641,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
+      <c r="A1" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="48.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="9" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>5</v>
@@ -2614,17 +2692,17 @@
     </row>
     <row r="4" spans="1:6" ht="81.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="9" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>5</v>
@@ -2632,19 +2710,19 @@
     </row>
     <row r="5" spans="1:6" ht="44.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="9" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>8</v>
@@ -2652,17 +2730,17 @@
     </row>
     <row r="6" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="9" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>8</v>
@@ -2670,17 +2748,17 @@
     </row>
     <row r="7" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>8</v>
@@ -2688,19 +2766,19 @@
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>11</v>
@@ -2708,461 +2786,461 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="9" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="9" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="9" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="9" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="9" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="9" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="9" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="9" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="9" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="9" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="9" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="9" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>216</v>
+        <v>175</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="9" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="9" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>216</v>
+        <v>175</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="9" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="9" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="9" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>228</v>
+        <v>198</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B33" s="9"/>
       <c r="C33" s="9" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>38</v>
@@ -3170,515 +3248,515 @@
     </row>
     <row r="34" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>228</v>
+        <v>166</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>228</v>
+        <v>169</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B38" s="9"/>
       <c r="C38" s="9" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B39" s="9"/>
       <c r="C39" s="9" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="67.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="9" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="9" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B41" s="9"/>
       <c r="C41" s="9" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="9" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="9" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B43" s="9"/>
       <c r="C43" s="9" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="9" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B44" s="9"/>
       <c r="C44" s="9" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B47" s="9"/>
       <c r="C47" s="9" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" s="9" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>258</v>
+        <v>157</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="9" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" s="9" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>258</v>
+        <v>234</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="67.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="9" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="9" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="9" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" s="9" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B54" s="9"/>
       <c r="C54" s="9" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B55" s="9"/>
       <c r="C55" s="9" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B56" s="9"/>
       <c r="C56" s="9" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="9" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B57" s="9"/>
       <c r="C57" s="9" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>271</v>
+        <v>234</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A58" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="B58" s="24"/>
-      <c r="C58" s="24"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
+      <c r="A58" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A59" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="B59" s="18" t="s">
-        <v>284</v>
-      </c>
-      <c r="C59" s="16"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="16"/>
-      <c r="F59" s="17"/>
+        <v>135</v>
+      </c>
+      <c r="B59" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A60" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B60" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="C60" s="16"/>
-      <c r="D60" s="16"/>
-      <c r="E60" s="16"/>
-      <c r="F60" s="17"/>
+        <v>136</v>
+      </c>
+      <c r="B60" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="16"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A61" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B61" s="18" t="s">
-        <v>286</v>
-      </c>
-      <c r="C61" s="16"/>
-      <c r="D61" s="16"/>
-      <c r="E61" s="16"/>
-      <c r="F61" s="17"/>
+        <v>64</v>
+      </c>
+      <c r="B61" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="16"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A62" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B62" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="C62" s="16"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="16"/>
-      <c r="F62" s="17"/>
+        <v>139</v>
+      </c>
+      <c r="B62" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="16"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A63" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="C63" s="16"/>
-      <c r="D63" s="16"/>
-      <c r="E63" s="16"/>
-      <c r="F63" s="17"/>
+        <v>283</v>
+      </c>
+      <c r="B63" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3701,259 +3779,283 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="19.25" style="8" customWidth="1"/>
-    <col min="3" max="3" width="50.25" style="8" customWidth="1"/>
+    <col min="2" max="2" width="42.375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="94.375" style="8" customWidth="1"/>
     <col min="4" max="4" width="35.125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
-        <v>290</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="135" x14ac:dyDescent="0.15">
-      <c r="A3" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="B3" s="14" t="s">
+    <row r="3" spans="1:4" ht="52.5" x14ac:dyDescent="0.15">
+      <c r="A3" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" ht="73.5" x14ac:dyDescent="0.15">
+      <c r="A4" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A5" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" ht="189" x14ac:dyDescent="0.15">
-      <c r="A4" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" s="14" t="s">
+      <c r="C6" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="52.5" x14ac:dyDescent="0.15">
+      <c r="A7" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" ht="135" x14ac:dyDescent="0.15">
-      <c r="A5" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="14" t="s">
+      <c r="C7" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A8" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="148.5" x14ac:dyDescent="0.15">
-      <c r="A6" s="14" t="s">
+      <c r="C8" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A9" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="D9" s="12"/>
+    </row>
+    <row r="10" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A10" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>300</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>301</v>
-      </c>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="B10" s="11" t="s">
         <v>303</v>
       </c>
-      <c r="D7" s="12"/>
-    </row>
-    <row r="8" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B8" s="14" t="s">
+      <c r="C10" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D10" s="12"/>
+    </row>
+    <row r="11" spans="1:4" ht="73.5" x14ac:dyDescent="0.15">
+      <c r="A11" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>305</v>
       </c>
-      <c r="D8" s="12"/>
-    </row>
-    <row r="9" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="B9" s="14" t="s">
+      <c r="C11" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D11" s="12"/>
+    </row>
+    <row r="12" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A12" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>307</v>
       </c>
-      <c r="D9" s="12"/>
-    </row>
-    <row r="10" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="B10" s="14" t="s">
+      <c r="C12" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A13" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>309</v>
       </c>
-      <c r="D10" s="12"/>
-    </row>
-    <row r="11" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="C13" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A14" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="D11" s="12"/>
-    </row>
-    <row r="12" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="B12" s="14" t="s">
+      <c r="C14" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D14" s="12"/>
+    </row>
+    <row r="15" spans="1:4" ht="52.5" x14ac:dyDescent="0.15">
+      <c r="A15" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="D12" s="12"/>
-    </row>
-    <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="B13" s="14" t="s">
+      <c r="C15" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="1:4" ht="84" x14ac:dyDescent="0.15">
+      <c r="A16" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="D13" s="12"/>
-    </row>
-    <row r="14" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="14" t="s">
-        <v>239</v>
-      </c>
-      <c r="B14" s="14" t="s">
+      <c r="C16" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A17" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B17" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="D14" s="12"/>
-    </row>
-    <row r="15" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="B15" s="14" t="s">
+      <c r="C17" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" spans="1:4" ht="73.5" x14ac:dyDescent="0.15">
+      <c r="A18" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="D15" s="12"/>
-    </row>
-    <row r="16" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="B16" s="14" t="s">
+      <c r="C18" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" spans="1:4" ht="52.5" x14ac:dyDescent="0.15">
+      <c r="A19" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="D16" s="12"/>
-    </row>
-    <row r="17" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="B17" s="14" t="s">
+      <c r="C19" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A20" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="D17" s="12"/>
-    </row>
-    <row r="18" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="B18" s="14" t="s">
+      <c r="C20" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A21" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" s="11" t="s">
         <v>325</v>
       </c>
-      <c r="D18" s="12"/>
-    </row>
-    <row r="19" spans="1:4" ht="283.5" x14ac:dyDescent="0.15">
-      <c r="A19" s="14" t="s">
-        <v>271</v>
-      </c>
-      <c r="B19" s="14" t="s">
+      <c r="C21" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="D21" s="12"/>
+    </row>
+    <row r="22" spans="1:4" ht="84" x14ac:dyDescent="0.15">
+      <c r="A22" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="D19" s="12"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="12"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="12"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="6"/>
+      <c r="C22" s="6" t="s">
+        <v>328</v>
+      </c>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="6"/>
+    <row r="23" spans="1:4" ht="63" x14ac:dyDescent="0.15">
+      <c r="A23" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
@@ -4179,44 +4281,44 @@
       <c r="D60" s="4"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A64" s="27" t="s">
-        <v>328</v>
-      </c>
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
+      <c r="A64" s="22" t="s">
+        <v>331</v>
+      </c>
+      <c r="B64" s="23"/>
+      <c r="C64" s="23"/>
+      <c r="D64" s="23"/>
     </row>
     <row r="65" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A65" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="B65" s="25" t="s">
-        <v>329</v>
-      </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="17"/>
+      <c r="A65" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="B65" s="26" t="s">
+        <v>332</v>
+      </c>
+      <c r="C65" s="15"/>
+      <c r="D65" s="16"/>
     </row>
     <row r="66" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A66" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="B66" s="25" t="s">
-        <v>330</v>
-      </c>
-      <c r="C66" s="16"/>
-      <c r="D66" s="17"/>
+      <c r="A66" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B66" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="C66" s="15"/>
+      <c r="D66" s="16"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A67" s="5"/>
-      <c r="B67" s="26"/>
-      <c r="C67" s="16"/>
-      <c r="D67" s="17"/>
+      <c r="B67" s="25"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="16"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A68" s="5"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="16"/>
-      <c r="D68" s="17"/>
+      <c r="B68" s="25"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4238,18 +4340,18 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="8" customWidth="1"/>
-    <col min="2" max="2" width="20" style="8" customWidth="1"/>
-    <col min="3" max="3" width="113.375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="31.75" style="8" customWidth="1"/>
+    <col min="3" max="3" width="103.75" style="8" customWidth="1"/>
     <col min="4" max="4" width="14.25" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -4265,280 +4367,250 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:4" ht="171" x14ac:dyDescent="0.15">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="256.5" x14ac:dyDescent="0.15">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:4" ht="207" x14ac:dyDescent="0.15">
+      <c r="A4" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="12"/>
     </row>
-    <row r="5" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:4" ht="252" x14ac:dyDescent="0.15">
+      <c r="A5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="12"/>
     </row>
-    <row r="6" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:4" ht="180" x14ac:dyDescent="0.15">
+      <c r="A6" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="12"/>
     </row>
-    <row r="7" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:4" ht="180" x14ac:dyDescent="0.15">
+      <c r="A7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="12"/>
     </row>
-    <row r="8" spans="1:4" ht="256.5" x14ac:dyDescent="0.15">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:4" ht="207" x14ac:dyDescent="0.15">
+      <c r="A8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="12"/>
     </row>
-    <row r="9" spans="1:4" ht="229.5" x14ac:dyDescent="0.15">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:4" ht="216" x14ac:dyDescent="0.15">
+      <c r="A9" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="12"/>
     </row>
-    <row r="10" spans="1:4" ht="324" x14ac:dyDescent="0.15">
-      <c r="A10" s="14" t="s">
+    <row r="10" spans="1:4" ht="189" x14ac:dyDescent="0.15">
+      <c r="A10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:4" ht="189" x14ac:dyDescent="0.15">
+      <c r="A11" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="3" t="s">
         <v>31</v>
       </c>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A12" s="14" t="s">
+    <row r="12" spans="1:4" ht="189" x14ac:dyDescent="0.15">
+      <c r="A12" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D12" s="12"/>
     </row>
-    <row r="13" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A13" s="14" t="s">
+    <row r="13" spans="1:4" ht="171" x14ac:dyDescent="0.15">
+      <c r="A13" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D13" s="12"/>
     </row>
-    <row r="14" spans="1:4" ht="175.5" x14ac:dyDescent="0.15">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:4" ht="252" x14ac:dyDescent="0.15">
+      <c r="A14" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D14" s="12"/>
     </row>
-    <row r="15" spans="1:4" ht="283.5" x14ac:dyDescent="0.15">
-      <c r="A15" s="14" t="s">
+    <row r="15" spans="1:4" ht="198" x14ac:dyDescent="0.15">
+      <c r="A15" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A16" s="14" t="s">
+    <row r="16" spans="1:4" ht="243" x14ac:dyDescent="0.15">
+      <c r="A16" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D16" s="12"/>
     </row>
-    <row r="17" spans="1:4" ht="297" x14ac:dyDescent="0.15">
-      <c r="A17" s="14" t="s">
+    <row r="17" spans="1:4" ht="189" x14ac:dyDescent="0.15">
+      <c r="A17" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D17" s="12"/>
     </row>
-    <row r="18" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:4" ht="180" x14ac:dyDescent="0.15">
+      <c r="A18" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="1:4" ht="243" x14ac:dyDescent="0.15">
-      <c r="A19" s="14" t="s">
+    <row r="19" spans="1:4" ht="261" x14ac:dyDescent="0.15">
+      <c r="A19" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="3" t="s">
         <v>55</v>
       </c>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A20" s="14" t="s">
+    <row r="20" spans="1:4" ht="171" x14ac:dyDescent="0.15">
+      <c r="A20" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="3" t="s">
         <v>58</v>
       </c>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A21" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>61</v>
-      </c>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="3"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="1:4" ht="297" x14ac:dyDescent="0.15">
-      <c r="A22" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>64</v>
-      </c>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="3"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" ht="216" x14ac:dyDescent="0.15">
-      <c r="A23" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>67</v>
-      </c>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="3"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="1:4" ht="202.5" x14ac:dyDescent="0.15">
-      <c r="A24" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>70</v>
-      </c>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="3"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="1:4" ht="364.5" x14ac:dyDescent="0.15">
-      <c r="A25" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>73</v>
-      </c>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="3"/>
       <c r="D25" s="12"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.15">

</xml_diff>